<commit_message>
Cierra punto pendiente de la auditoría de seguimiento v12: enlace de video y trazabilidad de commit en Anexo A
Agrega el informe de auditoría de seguimiento (7,9/10, aprobada con
observaciones menores). En Metadatos_corrida del Anexo A (Plantilla y
copia de rerun): reemplaza el placeholder pendiente por el enlace
público real a video_pretest.mov/video_postest.mov, y corrige el hash
de commit no trazable (911e07d) por una nota honesta que aclara que la
corrida se ejecutó sobre working tree local no commiteado, consolidado
después en el commit 97ce027.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Plantilla_Experimento_Pretest_Postest.xlsx
+++ b/docs/Plantilla_Experimento_Pretest_Postest.xlsx
@@ -2745,7 +2745,6 @@
         <v/>
       </c>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
@@ -3356,7 +3355,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>911e07d + cambios locales posteriores no commiteados: PedidoService.java (idempotencia + transicion atomica en cambiarEstado), PedidoRepository.java (marcarComoConfirmadoSiNoLoEstaba), PedidoFlowTest.java (test de regresion), docs/analisis/compute_stats.py (recalculo desde los rangos reales)</t>
+          <t>Working tree local no commiteado en el momento de la corrida (no corresponde a un commit del historial); los cambios se consolidaron despues en el commit 97ce027 del repositorio: PedidoService.java (idempotencia + transicion atomica en cambiarEstado), PedidoRepository.java (marcarComoConfirmadoSiNoLoEstaba), PedidoFlowTest.java (test de regresion), docs/analisis/compute_stats.py (recalculo desde los rangos reales)</t>
         </is>
       </c>
     </row>
@@ -3428,7 +3427,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>PENDIENTE: subir video_pretest.mov y video_postest.mov y pegar el enlace aca antes de la entrega</t>
+          <t>https://drive.google.com/drive/folders/1PkV-Dhm-Ba6JcGQq_6egg8op3uWXvSZN?usp=sharing</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Declara el historial de corridas y corrige los metadatos de la corrida
</commit_message>
<xml_diff>
--- a/docs/Plantilla_Experimento_Pretest_Postest.xlsx
+++ b/docs/Plantilla_Experimento_Pretest_Postest.xlsx
@@ -3550,7 +3550,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Working tree local no commiteado en el momento de la corrida (no corresponde a un commit del historial); los cambios se consolidaron despues en el commit 97ce027 del repositorio: PedidoService.java (idempotencia + transicion atomica en cambiarEstado), PedidoRepository.java (marcarComoConfirmadoSiNoLoEstaba), PedidoFlowTest.java (test de regresion), docs/analisis/compute_stats.py (recalculo desde los rangos reales)</t>
+          <t>Working tree local no commiteado en el momento de la corrida (no corresponde a un commit del historial). No se conserva registro de si ya incluia la correccion de concurrencia en la confirmacion de pedidos (PedidoService.java, PedidoRepository.java, PedidoFlowTest.java), que se consolido despues en el commit 97ce027 (13/09/2026).</t>
         </is>
       </c>
     </row>
@@ -3634,7 +3634,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>TPP y TED provienen de la corrida cronometrada y filmada (pretest 10/09, postest 12/09; instrumento unico: grabacion de pantalla con reloj visible, leido al segundo en ambas condiciones). Las correcciones de TED estan detalladas en la columna correspondiente de cada hoja (Pretest: escenarios 5 y 9; Postest: escenarios 8 y 14). NAS se verifico en una pasada suplementaria posterior (mismos 20 escenarios, sin video ni cronometraje) porque la base se reinicio por error antes de exportar el estado final de la corrida cronometrada; esa pasada tambien detecto y permitio corregir una condicion de carrera real en la confirmacion de pedidos (dos confirmaciones casi simultaneas sobre el mismo pedido descontaban stock dos veces), corregida en el codigo con una transaccion atomica en la base y verificada con 10 confirmaciones simultaneas de prueba. El pretest se cargo originalmente en formato a.m. por un default del editor de planillas; la corrida fue de noche (confirmado por la hora de guardado del video). Se sumaron 12 h a los horarios del pretest; los TPP (diferencias) no cambian.</t>
+          <t>TPP y TED provienen de la corrida cronometrada y filmada (pretest 10/09, postest 12/09; instrumento unico: grabacion de pantalla con reloj visible, leido al segundo en ambas condiciones). Las correcciones de TED estan detalladas en la columna correspondiente de cada hoja (Pretest: escenarios 5 y 9; Postest: escenarios 8 y 14). NAS se verifico en una pasada suplementaria posterior (mismos 20 escenarios, sin video ni cronometraje) porque la base se reinicio por error antes de exportar el estado final de la corrida cronometrada; el defecto de doble descuento de stock ante dos confirmaciones casi simultaneas sobre el mismo pedido se detecto en la pasada descartada del 11/09 y se corrigio con una transaccion atomica en la base (correccion verificada con 10 confirmaciones simultaneas de prueba); no se conserva registro de si la correccion ya estaba aplicada durante la corrida cronometrada. El pretest se cargo originalmente en formato a.m. por un default del editor de planillas; la corrida fue de noche (confirmado por la hora de guardado del video). Se sumaron 12 h a los horarios del pretest; los TPP (diferencias) no cambian.</t>
         </is>
       </c>
     </row>

</xml_diff>